<commit_message>
쿠팡 모니터링: coupang-monitoring-vercel 동기화 (결제 ~3/23, WAU 3/9주차)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Cursor/3_쿠팡 모니터링/cp_wau.xlsx
+++ b/Cursor/3_쿠팡 모니터링/cp_wau.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Cursor/3_쿠팡 모니터링/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Cursor/coupang-monitoring-vercel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E556EA60-470A-3346-8302-CA9AD65A1256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B01D5B-2F73-7B41-A43E-5195E98A1E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8160" yWindow="7200" windowWidth="27700" windowHeight="16880" xr2:uid="{557A2CCC-BB76-854E-B723-57C8CB621632}"/>
+    <workbookView xWindow="1940" yWindow="1340" windowWidth="27700" windowHeight="16880" xr2:uid="{557A2CCC-BB76-854E-B723-57C8CB621632}"/>
   </bookViews>
   <sheets>
     <sheet name="MI-INSIGHT1773654315714" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="48">
   <si>
     <t>모바일인덱스 INSIGHT CSV REPORT</t>
   </si>
@@ -161,6 +161,9 @@
   </si>
   <si>
     <t>2026-03-02 ~ 2026-03-08</t>
+  </si>
+  <si>
+    <t>2026-03-09 ~ 2026-03-15</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8398EB-50DF-6E4C-9081-89E2B7760E95}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1769,6 +1772,23 @@
         <v>8979524</v>
       </c>
     </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>10</v>
+      </c>
+      <c r="B44" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44">
+        <v>28281963</v>
+      </c>
+      <c r="D44">
+        <v>19347844</v>
+      </c>
+      <c r="E44">
+        <v>8934119</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>